<commit_message>
Separate encoding normalization from the SQL workflow
- Add a dedicated script to normalize corrupted French geographic labels
- Reorganize import validation and analysis scripts in execution order
- Preserve La Réunion metadata for consistent regional aggregation
- Refresh affected query screenshots with corrected accented labels
- Update the project documentation for the new four-step SQL workflow
</commit_message>
<xml_diff>
--- a/docs/data_dictionary.xlsx
+++ b/docs/data_dictionary.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elawy\Downloads\Divers\P4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elawy\Documents\DEV\assurance-habitation-sql\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{683B85BB-59AA-44B1-AA73-F097A241C529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F35290-059A-45E2-AA17-955BF2D57C21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -293,7 +293,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -342,90 +342,8 @@
       <left style="thick">
         <color rgb="FF833C0B"/>
       </left>
-      <right style="thick">
-        <color rgb="FF833C0B"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF833C0B"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF833C0B"/>
-      </left>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF833C0B"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF833C0B"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF833C0B"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF833C0B"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF833C0B"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF833C0B"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF833C0B"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF385623"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF385623"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF385623"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -441,83 +359,12 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thick">
-        <color rgb="FF385623"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF385623"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF385623"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF385623"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF385623"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thick">
         <color rgb="FF385623"/>
       </left>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF385623"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF385623"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF385623"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF385623"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF385623"/>
-      </right>
-      <top/>
-      <bottom style="thick">
-        <color rgb="FF385623"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -532,20 +379,56 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thick">
+        <color rgb="FF833C0B"/>
+      </left>
       <right/>
-      <top/>
-      <bottom style="thick">
-        <color rgb="FF385623"/>
+      <top style="thick">
+        <color rgb="FF833C0B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1E4E79"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1E4E79"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF1E4E79"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1E4E79"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thick">
-        <color rgb="FF385623"/>
+      <left style="medium">
+        <color rgb="FF1E4E79"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1E4E79"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color rgb="FF1E4E79"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1E4E79"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1E4E79"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1E4E79"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1E4E79"/>
+      </top>
       <bottom style="thick">
         <color rgb="FF385623"/>
       </bottom>
@@ -555,11 +438,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -569,98 +449,79 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -891,1132 +752,1132 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="34"/>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
-      <c r="L1" s="34"/>
-      <c r="M1" s="34"/>
-      <c r="N1" s="34"/>
-      <c r="O1" s="34"/>
-      <c r="P1" s="34"/>
+      <c r="A1" s="4"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="34"/>
-      <c r="B2" s="35"/>
-      <c r="C2" s="2" t="s">
+      <c r="A2" s="4"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
-      <c r="M2" s="34"/>
-      <c r="N2" s="34"/>
-      <c r="O2" s="34"/>
-      <c r="P2" s="34"/>
-    </row>
-    <row r="3" spans="1:16" ht="24.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="34"/>
-      <c r="B3" s="14" t="s">
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+    </row>
+    <row r="3" spans="1:16" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4"/>
+      <c r="B3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="23"/>
-      <c r="F3" s="1" t="s">
+      <c r="E3" s="13"/>
+      <c r="F3" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
-      <c r="K3" s="34"/>
-      <c r="L3" s="34"/>
-      <c r="M3" s="34"/>
-      <c r="N3" s="34"/>
-      <c r="O3" s="34"/>
-      <c r="P3" s="34"/>
-    </row>
-    <row r="4" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="34"/>
-      <c r="B4" s="15"/>
-      <c r="C4" s="39" t="s">
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+    </row>
+    <row r="4" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="4"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="16">
         <v>10</v>
       </c>
-      <c r="F4" s="24"/>
-      <c r="G4" s="29" t="s">
+      <c r="F4" s="17"/>
+      <c r="G4" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="34"/>
-      <c r="M4" s="34"/>
-      <c r="N4" s="34"/>
-      <c r="O4" s="34"/>
-      <c r="P4" s="34"/>
-    </row>
-    <row r="5" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="34"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="5" t="s">
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+    </row>
+    <row r="5" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="23">
+      <c r="E5" s="20">
         <v>1</v>
       </c>
-      <c r="F5" s="1"/>
-      <c r="G5" s="28" t="s">
+      <c r="F5" s="19"/>
+      <c r="G5" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="34"/>
-      <c r="I5" s="34"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="34"/>
-      <c r="N5" s="34"/>
-      <c r="O5" s="34"/>
-      <c r="P5" s="34"/>
-    </row>
-    <row r="6" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="34"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="6" t="s">
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+    </row>
+    <row r="6" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="16">
         <v>10</v>
       </c>
-      <c r="F6" s="24"/>
-      <c r="G6" s="30" t="s">
+      <c r="F6" s="17"/>
+      <c r="G6" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="34"/>
-      <c r="M6" s="34"/>
-      <c r="N6" s="34"/>
-      <c r="O6" s="34"/>
-      <c r="P6" s="34"/>
-    </row>
-    <row r="7" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="34"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="5" t="s">
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+    </row>
+    <row r="7" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="38" t="s">
+      <c r="D7" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="20">
         <v>100</v>
       </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="28" t="s">
+      <c r="F7" s="19"/>
+      <c r="G7" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="34"/>
-      <c r="I7" s="34"/>
-      <c r="J7" s="34"/>
-      <c r="K7" s="34"/>
-      <c r="L7" s="34"/>
-      <c r="M7" s="34"/>
-      <c r="N7" s="34"/>
-      <c r="O7" s="34"/>
-      <c r="P7" s="34"/>
-    </row>
-    <row r="8" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="34"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="6" t="s">
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+    </row>
+    <row r="8" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="25">
+      <c r="E8" s="24">
         <v>6</v>
       </c>
-      <c r="F8" s="37" t="s">
+      <c r="F8" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="G8" s="30" t="s">
+      <c r="G8" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
-      <c r="J8" s="34"/>
-      <c r="K8" s="34"/>
-      <c r="L8" s="34"/>
-      <c r="M8" s="34"/>
-      <c r="N8" s="34"/>
-      <c r="O8" s="34"/>
-      <c r="P8" s="34"/>
-    </row>
-    <row r="9" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="34"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="5" t="s">
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+    </row>
+    <row r="9" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="4"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="19">
         <v>5</v>
       </c>
-      <c r="F9" s="26"/>
-      <c r="G9" s="31" t="s">
+      <c r="F9" s="25"/>
+      <c r="G9" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="34"/>
-      <c r="I9" s="34"/>
-      <c r="J9" s="34"/>
-      <c r="K9" s="34"/>
-      <c r="L9" s="34"/>
-      <c r="M9" s="34"/>
-      <c r="N9" s="34"/>
-      <c r="O9" s="34"/>
-      <c r="P9" s="34"/>
-    </row>
-    <row r="10" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="34"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="6" t="s">
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+    </row>
+    <row r="10" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="4"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="E10" s="25"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="30" t="s">
+      <c r="E10" s="24"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="H10" s="34"/>
-      <c r="I10" s="34"/>
-      <c r="J10" s="34"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="34"/>
-      <c r="M10" s="34"/>
-      <c r="N10" s="34"/>
-      <c r="O10" s="34"/>
-      <c r="P10" s="34"/>
-    </row>
-    <row r="11" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="34"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="22" t="s">
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+    </row>
+    <row r="11" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="4"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="19">
         <v>30</v>
       </c>
-      <c r="F11" s="26"/>
-      <c r="G11" s="28" t="s">
+      <c r="F11" s="25"/>
+      <c r="G11" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="H11" s="34"/>
-      <c r="I11" s="34"/>
-      <c r="J11" s="34"/>
-      <c r="K11" s="34"/>
-      <c r="L11" s="34"/>
-      <c r="M11" s="34"/>
-      <c r="N11" s="34"/>
-      <c r="O11" s="34"/>
-      <c r="P11" s="34"/>
-    </row>
-    <row r="12" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="34"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="6" t="s">
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4"/>
+    </row>
+    <row r="12" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="4"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="24">
         <v>30</v>
       </c>
-      <c r="F12" s="7"/>
-      <c r="G12" s="30" t="s">
+      <c r="F12" s="16"/>
+      <c r="G12" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="H12" s="34"/>
-      <c r="I12" s="34"/>
-      <c r="J12" s="34"/>
-      <c r="K12" s="34"/>
-      <c r="L12" s="34"/>
-      <c r="M12" s="34"/>
-      <c r="N12" s="34"/>
-      <c r="O12" s="34"/>
-      <c r="P12" s="34"/>
-    </row>
-    <row r="13" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="34"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="5" t="s">
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+    </row>
+    <row r="13" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="4"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="19">
         <v>40</v>
       </c>
-      <c r="F13" s="26"/>
-      <c r="G13" s="31" t="s">
+      <c r="F13" s="25"/>
+      <c r="G13" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="H13" s="34"/>
-      <c r="I13" s="34"/>
-      <c r="J13" s="34"/>
-      <c r="K13" s="34"/>
-      <c r="L13" s="34"/>
-      <c r="M13" s="34"/>
-      <c r="N13" s="34"/>
-      <c r="O13" s="34"/>
-      <c r="P13" s="34"/>
-    </row>
-    <row r="14" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="34"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="6" t="s">
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4"/>
+    </row>
+    <row r="14" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="4"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="25">
+      <c r="E14" s="24">
         <v>30</v>
       </c>
-      <c r="F14" s="7"/>
-      <c r="G14" s="30" t="s">
+      <c r="F14" s="16"/>
+      <c r="G14" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="H14" s="34"/>
-      <c r="I14" s="34"/>
-      <c r="J14" s="34"/>
-      <c r="K14" s="34"/>
-      <c r="L14" s="34"/>
-      <c r="M14" s="34"/>
-      <c r="N14" s="34"/>
-      <c r="O14" s="34"/>
-      <c r="P14" s="34"/>
-    </row>
-    <row r="15" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="34"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="5" t="s">
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="4"/>
+    </row>
+    <row r="15" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="4"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="19">
         <v>30</v>
       </c>
-      <c r="F15" s="26"/>
-      <c r="G15" s="31" t="s">
+      <c r="F15" s="25"/>
+      <c r="G15" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="H15" s="34"/>
-      <c r="I15" s="34"/>
-      <c r="J15" s="34"/>
-      <c r="K15" s="34"/>
-      <c r="L15" s="34"/>
-      <c r="M15" s="34"/>
-      <c r="N15" s="34"/>
-      <c r="O15" s="34"/>
-      <c r="P15" s="34"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4"/>
     </row>
     <row r="16" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="34"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="6" t="s">
+      <c r="A16" s="4"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="D16" s="37" t="s">
+      <c r="D16" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="25">
+      <c r="E16" s="24">
         <v>10.199999999999999</v>
       </c>
-      <c r="F16" s="7"/>
-      <c r="G16" s="29" t="s">
+      <c r="F16" s="16"/>
+      <c r="G16" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="H16" s="34"/>
-      <c r="I16" s="34"/>
-      <c r="J16" s="34"/>
-      <c r="K16" s="34"/>
-      <c r="L16" s="34"/>
-      <c r="M16" s="34"/>
-      <c r="N16" s="34"/>
-      <c r="O16" s="34"/>
-      <c r="P16" s="34"/>
-    </row>
-    <row r="17" spans="1:16" ht="24.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="34"/>
-      <c r="B17" s="17" t="s">
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="4"/>
+    </row>
+    <row r="17" spans="1:16" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="4"/>
+      <c r="B17" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="D17" s="27" t="s">
+      <c r="D17" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="27">
+      <c r="E17" s="19">
         <v>6</v>
       </c>
-      <c r="F17" s="27" t="s">
+      <c r="F17" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="32" t="s">
+      <c r="G17" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="H17" s="34"/>
-      <c r="I17" s="34"/>
-      <c r="J17" s="34"/>
-      <c r="K17" s="34"/>
-      <c r="L17" s="34"/>
-      <c r="M17" s="34"/>
-      <c r="N17" s="34"/>
-      <c r="O17" s="34"/>
-      <c r="P17" s="34"/>
-    </row>
-    <row r="18" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="34"/>
-      <c r="B18" s="18"/>
-      <c r="C18" s="8" t="s">
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="4"/>
+    </row>
+    <row r="18" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="28">
         <v>2</v>
       </c>
-      <c r="F18" s="9"/>
-      <c r="G18" s="10" t="s">
+      <c r="F18" s="28"/>
+      <c r="G18" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="H18" s="34"/>
-      <c r="I18" s="34"/>
-      <c r="J18" s="34"/>
-      <c r="K18" s="34"/>
-      <c r="L18" s="34"/>
-      <c r="M18" s="34"/>
-      <c r="N18" s="34"/>
-      <c r="O18" s="34"/>
-      <c r="P18" s="34"/>
-    </row>
-    <row r="19" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="34"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="21" t="s">
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="4"/>
+    </row>
+    <row r="19" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="4"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="19">
         <v>50</v>
       </c>
-      <c r="F19" s="1"/>
-      <c r="G19" s="33" t="s">
+      <c r="F19" s="19"/>
+      <c r="G19" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="H19" s="34"/>
-      <c r="I19" s="34"/>
-      <c r="J19" s="34"/>
-      <c r="K19" s="34"/>
-      <c r="L19" s="34"/>
-      <c r="M19" s="34"/>
-      <c r="N19" s="34"/>
-      <c r="O19" s="34"/>
-      <c r="P19" s="34"/>
-    </row>
-    <row r="20" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="34"/>
-      <c r="B20" s="18"/>
-      <c r="C20" s="8" t="s">
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4"/>
+    </row>
+    <row r="20" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="4"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20" s="28">
         <v>50</v>
       </c>
-      <c r="F20" s="9"/>
-      <c r="G20" s="10" t="s">
+      <c r="F20" s="28"/>
+      <c r="G20" s="29" t="s">
         <v>49</v>
       </c>
-      <c r="H20" s="34"/>
-      <c r="I20" s="34"/>
-      <c r="J20" s="34"/>
-      <c r="K20" s="34"/>
-      <c r="L20" s="34"/>
-      <c r="M20" s="34"/>
-      <c r="N20" s="34"/>
-      <c r="O20" s="34"/>
-      <c r="P20" s="34"/>
-    </row>
-    <row r="21" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="34"/>
-      <c r="B21" s="18"/>
-      <c r="C21" s="21" t="s">
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="4"/>
+    </row>
+    <row r="21" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="4"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="19">
         <v>60</v>
       </c>
-      <c r="F21" s="1"/>
-      <c r="G21" s="33" t="s">
+      <c r="F21" s="19"/>
+      <c r="G21" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="H21" s="34"/>
-      <c r="I21" s="34"/>
-      <c r="J21" s="34"/>
-      <c r="K21" s="34"/>
-      <c r="L21" s="34"/>
-      <c r="M21" s="34"/>
-      <c r="N21" s="34"/>
-      <c r="O21" s="34"/>
-      <c r="P21" s="34"/>
-    </row>
-    <row r="22" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="34"/>
-      <c r="B22" s="18"/>
-      <c r="C22" s="8" t="s">
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="4"/>
+    </row>
+    <row r="22" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="4"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="E22" s="9">
+      <c r="E22" s="28">
         <v>80</v>
       </c>
-      <c r="F22" s="9"/>
-      <c r="G22" s="10" t="s">
+      <c r="F22" s="28"/>
+      <c r="G22" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="H22" s="34"/>
-      <c r="I22" s="34"/>
-      <c r="J22" s="34"/>
-      <c r="K22" s="34"/>
-      <c r="L22" s="34"/>
-      <c r="M22" s="34"/>
-      <c r="N22" s="34"/>
-      <c r="O22" s="34"/>
-      <c r="P22" s="34"/>
-    </row>
-    <row r="23" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="34"/>
-      <c r="B23" s="18"/>
-      <c r="C23" s="21" t="s">
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="4"/>
+    </row>
+    <row r="23" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="4"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="19">
         <v>3</v>
       </c>
-      <c r="F23" s="1"/>
-      <c r="G23" s="33" t="s">
+      <c r="F23" s="19"/>
+      <c r="G23" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="H23" s="34"/>
-      <c r="I23" s="34"/>
-      <c r="J23" s="34"/>
-      <c r="K23" s="34"/>
-      <c r="L23" s="34"/>
-      <c r="M23" s="34"/>
-      <c r="N23" s="34"/>
-      <c r="O23" s="34"/>
-      <c r="P23" s="34"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4"/>
+      <c r="P23" s="4"/>
     </row>
     <row r="24" spans="1:16" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="34"/>
-      <c r="B24" s="19"/>
-      <c r="C24" s="11" t="s">
+      <c r="A24" s="4"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="D24" s="12" t="s">
+      <c r="D24" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="30">
         <v>80</v>
       </c>
-      <c r="F24" s="12"/>
-      <c r="G24" s="13" t="s">
+      <c r="F24" s="30"/>
+      <c r="G24" s="31" t="s">
         <v>53</v>
       </c>
-      <c r="H24" s="34"/>
-      <c r="I24" s="34"/>
-      <c r="J24" s="34"/>
-      <c r="K24" s="34"/>
-      <c r="L24" s="34"/>
-      <c r="M24" s="34"/>
-      <c r="N24" s="34"/>
-      <c r="O24" s="34"/>
-      <c r="P24" s="34"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4"/>
     </row>
     <row r="25" spans="1:16" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="34"/>
-      <c r="B25" s="34"/>
-      <c r="C25" s="34"/>
-      <c r="D25" s="34"/>
-      <c r="E25" s="34"/>
-      <c r="F25" s="34"/>
-      <c r="G25" s="34"/>
-      <c r="H25" s="34"/>
-      <c r="I25" s="34"/>
-      <c r="J25" s="34"/>
-      <c r="K25" s="34"/>
-      <c r="L25" s="34"/>
-      <c r="M25" s="34"/>
-      <c r="N25" s="34"/>
-      <c r="O25" s="34"/>
-      <c r="P25" s="34"/>
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="4"/>
     </row>
     <row r="26" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="34"/>
-      <c r="B26" s="34"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="34"/>
-      <c r="F26" s="34"/>
-      <c r="G26" s="34"/>
-      <c r="H26" s="34"/>
-      <c r="I26" s="34"/>
-      <c r="J26" s="34"/>
-      <c r="K26" s="34"/>
-      <c r="L26" s="34"/>
-      <c r="M26" s="34"/>
-      <c r="N26" s="34"/>
-      <c r="O26" s="34"/>
-      <c r="P26" s="34"/>
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="L26" s="4"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4"/>
+      <c r="O26" s="4"/>
+      <c r="P26" s="4"/>
     </row>
     <row r="27" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="34"/>
-      <c r="B27" s="34"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="34"/>
-      <c r="F27" s="34"/>
-      <c r="G27" s="34"/>
-      <c r="H27" s="34"/>
-      <c r="I27" s="34"/>
-      <c r="J27" s="34"/>
-      <c r="K27" s="34"/>
-      <c r="L27" s="34"/>
-      <c r="M27" s="34"/>
-      <c r="N27" s="34"/>
-      <c r="O27" s="34"/>
-      <c r="P27" s="34"/>
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+      <c r="O27" s="4"/>
+      <c r="P27" s="4"/>
     </row>
     <row r="28" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="34"/>
-      <c r="B28" s="34"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="34"/>
-      <c r="E28" s="34"/>
-      <c r="F28" s="34"/>
-      <c r="G28" s="34"/>
-      <c r="H28" s="34"/>
-      <c r="I28" s="34"/>
-      <c r="J28" s="34"/>
-      <c r="K28" s="34"/>
-      <c r="L28" s="34"/>
-      <c r="M28" s="34"/>
-      <c r="N28" s="34"/>
-      <c r="O28" s="34"/>
-      <c r="P28" s="34"/>
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4"/>
+      <c r="O28" s="4"/>
+      <c r="P28" s="4"/>
     </row>
     <row r="29" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="34"/>
-      <c r="B29" s="34"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="34"/>
-      <c r="E29" s="34"/>
-      <c r="F29" s="34"/>
-      <c r="G29" s="34"/>
-      <c r="H29" s="34"/>
-      <c r="I29" s="34"/>
-      <c r="J29" s="34"/>
-      <c r="K29" s="34"/>
-      <c r="L29" s="34"/>
-      <c r="M29" s="34"/>
-      <c r="N29" s="34"/>
-      <c r="O29" s="34"/>
-      <c r="P29" s="34"/>
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4"/>
+      <c r="O29" s="4"/>
+      <c r="P29" s="4"/>
     </row>
     <row r="30" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="34"/>
-      <c r="B30" s="34"/>
-      <c r="C30" s="34"/>
-      <c r="D30" s="34"/>
-      <c r="E30" s="34"/>
-      <c r="F30" s="34"/>
-      <c r="G30" s="34"/>
-      <c r="H30" s="34"/>
-      <c r="I30" s="34"/>
-      <c r="J30" s="34"/>
-      <c r="K30" s="34"/>
-      <c r="L30" s="34"/>
-      <c r="M30" s="34"/>
-      <c r="N30" s="34"/>
-      <c r="O30" s="34"/>
-      <c r="P30" s="34"/>
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4"/>
+      <c r="L30" s="4"/>
+      <c r="M30" s="4"/>
+      <c r="N30" s="4"/>
+      <c r="O30" s="4"/>
+      <c r="P30" s="4"/>
     </row>
     <row r="31" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="34"/>
-      <c r="B31" s="34"/>
-      <c r="C31" s="34"/>
-      <c r="D31" s="34"/>
-      <c r="E31" s="34"/>
-      <c r="F31" s="34"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="34"/>
-      <c r="I31" s="34"/>
-      <c r="J31" s="34"/>
-      <c r="K31" s="34"/>
-      <c r="L31" s="34"/>
-      <c r="M31" s="34"/>
-      <c r="N31" s="34"/>
-      <c r="O31" s="34"/>
-      <c r="P31" s="34"/>
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
+      <c r="I31" s="4"/>
+      <c r="J31" s="4"/>
+      <c r="K31" s="4"/>
+      <c r="L31" s="4"/>
+      <c r="M31" s="4"/>
+      <c r="N31" s="4"/>
+      <c r="O31" s="4"/>
+      <c r="P31" s="4"/>
     </row>
     <row r="32" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="34"/>
-      <c r="B32" s="34"/>
-      <c r="C32" s="34"/>
-      <c r="D32" s="34"/>
-      <c r="E32" s="34"/>
-      <c r="F32" s="34"/>
-      <c r="G32" s="34"/>
-      <c r="H32" s="34"/>
-      <c r="I32" s="34"/>
-      <c r="J32" s="34"/>
-      <c r="K32" s="34"/>
-      <c r="L32" s="34"/>
-      <c r="M32" s="34"/>
-      <c r="N32" s="34"/>
-      <c r="O32" s="34"/>
-      <c r="P32" s="34"/>
+      <c r="A32" s="4"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4"/>
+      <c r="L32" s="4"/>
+      <c r="M32" s="4"/>
+      <c r="N32" s="4"/>
+      <c r="O32" s="4"/>
+      <c r="P32" s="4"/>
     </row>
     <row r="33" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="34"/>
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="34"/>
-      <c r="G33" s="34"/>
-      <c r="H33" s="34"/>
-      <c r="I33" s="34"/>
-      <c r="J33" s="34"/>
-      <c r="K33" s="34"/>
-      <c r="L33" s="34"/>
-      <c r="M33" s="34"/>
-      <c r="N33" s="34"/>
-      <c r="O33" s="34"/>
-      <c r="P33" s="34"/>
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
+      <c r="L33" s="4"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="4"/>
+      <c r="O33" s="4"/>
+      <c r="P33" s="4"/>
     </row>
     <row r="34" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="34"/>
-      <c r="B34" s="34"/>
-      <c r="C34" s="34"/>
-      <c r="D34" s="34"/>
-      <c r="E34" s="34"/>
-      <c r="F34" s="34"/>
-      <c r="G34" s="34"/>
-      <c r="H34" s="34"/>
-      <c r="I34" s="34"/>
-      <c r="J34" s="34"/>
-      <c r="K34" s="34"/>
-      <c r="L34" s="34"/>
-      <c r="M34" s="34"/>
-      <c r="N34" s="34"/>
-      <c r="O34" s="34"/>
-      <c r="P34" s="34"/>
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4"/>
+      <c r="L34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
+      <c r="P34" s="4"/>
     </row>
     <row r="35" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="34"/>
-      <c r="B35" s="34"/>
-      <c r="C35" s="34"/>
-      <c r="D35" s="34"/>
-      <c r="E35" s="34"/>
-      <c r="F35" s="34"/>
-      <c r="G35" s="34"/>
-      <c r="H35" s="34"/>
-      <c r="I35" s="34"/>
-      <c r="J35" s="34"/>
-      <c r="K35" s="34"/>
-      <c r="L35" s="34"/>
-      <c r="M35" s="34"/>
-      <c r="N35" s="34"/>
-      <c r="O35" s="34"/>
-      <c r="P35" s="34"/>
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
+      <c r="I35" s="4"/>
+      <c r="J35" s="4"/>
+      <c r="K35" s="4"/>
+      <c r="L35" s="4"/>
+      <c r="M35" s="4"/>
+      <c r="N35" s="4"/>
+      <c r="O35" s="4"/>
+      <c r="P35" s="4"/>
     </row>
     <row r="36" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="34"/>
-      <c r="B36" s="34"/>
-      <c r="C36" s="34"/>
-      <c r="D36" s="34"/>
-      <c r="E36" s="34"/>
-      <c r="F36" s="34"/>
-      <c r="G36" s="34"/>
-      <c r="H36" s="34"/>
-      <c r="I36" s="34"/>
-      <c r="J36" s="34"/>
-      <c r="K36" s="34"/>
-      <c r="L36" s="34"/>
-      <c r="M36" s="34"/>
-      <c r="N36" s="34"/>
-      <c r="O36" s="34"/>
-      <c r="P36" s="34"/>
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4"/>
+      <c r="I36" s="4"/>
+      <c r="J36" s="4"/>
+      <c r="K36" s="4"/>
+      <c r="L36" s="4"/>
+      <c r="M36" s="4"/>
+      <c r="N36" s="4"/>
+      <c r="O36" s="4"/>
+      <c r="P36" s="4"/>
     </row>
     <row r="37" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="34"/>
-      <c r="B37" s="34"/>
-      <c r="C37" s="34"/>
-      <c r="D37" s="34"/>
-      <c r="E37" s="34"/>
-      <c r="F37" s="34"/>
-      <c r="G37" s="34"/>
-      <c r="H37" s="34"/>
-      <c r="I37" s="34"/>
-      <c r="J37" s="34"/>
-      <c r="K37" s="34"/>
-      <c r="L37" s="34"/>
-      <c r="M37" s="34"/>
-      <c r="N37" s="34"/>
-      <c r="O37" s="34"/>
-      <c r="P37" s="34"/>
+      <c r="A37" s="4"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="4"/>
+      <c r="I37" s="4"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4"/>
+      <c r="L37" s="4"/>
+      <c r="M37" s="4"/>
+      <c r="N37" s="4"/>
+      <c r="O37" s="4"/>
+      <c r="P37" s="4"/>
     </row>
     <row r="38" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="34"/>
-      <c r="B38" s="34"/>
-      <c r="C38" s="34"/>
-      <c r="D38" s="34"/>
-      <c r="E38" s="34"/>
-      <c r="F38" s="34"/>
-      <c r="G38" s="34"/>
-      <c r="H38" s="34"/>
-      <c r="I38" s="34"/>
-      <c r="J38" s="34"/>
-      <c r="K38" s="34"/>
-      <c r="L38" s="34"/>
-      <c r="M38" s="34"/>
-      <c r="N38" s="34"/>
-      <c r="O38" s="34"/>
-      <c r="P38" s="34"/>
+      <c r="A38" s="4"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
+      <c r="I38" s="4"/>
+      <c r="J38" s="4"/>
+      <c r="K38" s="4"/>
+      <c r="L38" s="4"/>
+      <c r="M38" s="4"/>
+      <c r="N38" s="4"/>
+      <c r="O38" s="4"/>
+      <c r="P38" s="4"/>
     </row>
     <row r="39" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="34"/>
-      <c r="B39" s="34"/>
-      <c r="C39" s="34"/>
-      <c r="D39" s="34"/>
-      <c r="E39" s="34"/>
-      <c r="F39" s="34"/>
-      <c r="G39" s="34"/>
-      <c r="H39" s="34"/>
-      <c r="I39" s="34"/>
-      <c r="J39" s="34"/>
-      <c r="K39" s="34"/>
-      <c r="L39" s="34"/>
-      <c r="M39" s="34"/>
-      <c r="N39" s="34"/>
-      <c r="O39" s="34"/>
-      <c r="P39" s="34"/>
+      <c r="A39" s="4"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="4"/>
+      <c r="K39" s="4"/>
+      <c r="L39" s="4"/>
+      <c r="M39" s="4"/>
+      <c r="N39" s="4"/>
+      <c r="O39" s="4"/>
+      <c r="P39" s="4"/>
     </row>
     <row r="40" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="34"/>
-      <c r="B40" s="34"/>
-      <c r="C40" s="34"/>
-      <c r="D40" s="34"/>
-      <c r="E40" s="34"/>
-      <c r="F40" s="34"/>
-      <c r="G40" s="34"/>
-      <c r="H40" s="34"/>
-      <c r="I40" s="34"/>
-      <c r="J40" s="34"/>
-      <c r="K40" s="34"/>
-      <c r="L40" s="34"/>
-      <c r="M40" s="34"/>
-      <c r="N40" s="34"/>
-      <c r="O40" s="34"/>
-      <c r="P40" s="34"/>
+      <c r="A40" s="4"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4"/>
+      <c r="K40" s="4"/>
+      <c r="L40" s="4"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="4"/>
+      <c r="O40" s="4"/>
+      <c r="P40" s="4"/>
     </row>
     <row r="41" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="34"/>
-      <c r="B41" s="34"/>
-      <c r="C41" s="34"/>
-      <c r="D41" s="34"/>
-      <c r="E41" s="34"/>
-      <c r="F41" s="34"/>
-      <c r="G41" s="34"/>
-      <c r="H41" s="34"/>
-      <c r="I41" s="34"/>
-      <c r="J41" s="34"/>
-      <c r="K41" s="34"/>
-      <c r="L41" s="34"/>
-      <c r="M41" s="34"/>
-      <c r="N41" s="34"/>
-      <c r="O41" s="34"/>
-      <c r="P41" s="34"/>
+      <c r="A41" s="4"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4"/>
+      <c r="I41" s="4"/>
+      <c r="J41" s="4"/>
+      <c r="K41" s="4"/>
+      <c r="L41" s="4"/>
+      <c r="M41" s="4"/>
+      <c r="N41" s="4"/>
+      <c r="O41" s="4"/>
+      <c r="P41" s="4"/>
     </row>
     <row r="42" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="34"/>
-      <c r="B42" s="34"/>
-      <c r="C42" s="34"/>
-      <c r="D42" s="34"/>
-      <c r="E42" s="34"/>
-      <c r="F42" s="34"/>
-      <c r="G42" s="34"/>
-      <c r="H42" s="34"/>
-      <c r="I42" s="34"/>
-      <c r="J42" s="34"/>
-      <c r="K42" s="34"/>
-      <c r="L42" s="34"/>
-      <c r="M42" s="34"/>
-      <c r="N42" s="34"/>
-      <c r="O42" s="34"/>
-      <c r="P42" s="34"/>
+      <c r="A42" s="4"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="4"/>
+      <c r="L42" s="4"/>
+      <c r="M42" s="4"/>
+      <c r="N42" s="4"/>
+      <c r="O42" s="4"/>
+      <c r="P42" s="4"/>
     </row>
     <row r="43" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="34"/>
-      <c r="B43" s="34"/>
-      <c r="C43" s="34"/>
-      <c r="D43" s="34"/>
-      <c r="E43" s="34"/>
-      <c r="F43" s="34"/>
-      <c r="G43" s="34"/>
-      <c r="H43" s="34"/>
-      <c r="I43" s="34"/>
-      <c r="J43" s="34"/>
-      <c r="K43" s="34"/>
-      <c r="L43" s="34"/>
-      <c r="M43" s="34"/>
-      <c r="N43" s="34"/>
-      <c r="O43" s="34"/>
-      <c r="P43" s="34"/>
+      <c r="A43" s="4"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
+      <c r="G43" s="4"/>
+      <c r="H43" s="4"/>
+      <c r="I43" s="4"/>
+      <c r="J43" s="4"/>
+      <c r="K43" s="4"/>
+      <c r="L43" s="4"/>
+      <c r="M43" s="4"/>
+      <c r="N43" s="4"/>
+      <c r="O43" s="4"/>
+      <c r="P43" s="4"/>
     </row>
     <row r="44" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="34"/>
-      <c r="B44" s="34"/>
-      <c r="C44" s="34"/>
-      <c r="D44" s="34"/>
-      <c r="E44" s="34"/>
-      <c r="F44" s="34"/>
-      <c r="G44" s="34"/>
-      <c r="H44" s="34"/>
-      <c r="I44" s="34"/>
-      <c r="J44" s="34"/>
-      <c r="K44" s="34"/>
-      <c r="L44" s="34"/>
-      <c r="M44" s="34"/>
-      <c r="N44" s="34"/>
-      <c r="O44" s="34"/>
-      <c r="P44" s="34"/>
+      <c r="A44" s="4"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4"/>
+      <c r="H44" s="4"/>
+      <c r="I44" s="4"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="4"/>
+      <c r="L44" s="4"/>
+      <c r="M44" s="4"/>
+      <c r="N44" s="4"/>
+      <c r="O44" s="4"/>
+      <c r="P44" s="4"/>
     </row>
     <row r="45" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="34"/>
-      <c r="B45" s="34"/>
-      <c r="C45" s="34"/>
-      <c r="D45" s="34"/>
-      <c r="E45" s="34"/>
-      <c r="F45" s="34"/>
-      <c r="G45" s="34"/>
-      <c r="H45" s="34"/>
-      <c r="I45" s="34"/>
-      <c r="J45" s="34"/>
-      <c r="K45" s="34"/>
-      <c r="L45" s="34"/>
-      <c r="M45" s="34"/>
-      <c r="N45" s="34"/>
-      <c r="O45" s="34"/>
-      <c r="P45" s="34"/>
+      <c r="A45" s="4"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4"/>
+      <c r="I45" s="4"/>
+      <c r="J45" s="4"/>
+      <c r="K45" s="4"/>
+      <c r="L45" s="4"/>
+      <c r="M45" s="4"/>
+      <c r="N45" s="4"/>
+      <c r="O45" s="4"/>
+      <c r="P45" s="4"/>
     </row>
     <row r="46" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="34"/>
-      <c r="B46" s="34"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="34"/>
-      <c r="E46" s="34"/>
-      <c r="F46" s="34"/>
-      <c r="G46" s="34"/>
-      <c r="H46" s="34"/>
-      <c r="I46" s="34"/>
-      <c r="J46" s="34"/>
-      <c r="K46" s="34"/>
-      <c r="L46" s="34"/>
-      <c r="M46" s="34"/>
-      <c r="N46" s="34"/>
-      <c r="O46" s="34"/>
-      <c r="P46" s="34"/>
+      <c r="A46" s="4"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="4"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="4"/>
+      <c r="L46" s="4"/>
+      <c r="M46" s="4"/>
+      <c r="N46" s="4"/>
+      <c r="O46" s="4"/>
+      <c r="P46" s="4"/>
     </row>
     <row r="47" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="34"/>
-      <c r="B47" s="34"/>
-      <c r="C47" s="34"/>
-      <c r="D47" s="34"/>
-      <c r="E47" s="34"/>
-      <c r="F47" s="34"/>
-      <c r="G47" s="34"/>
-      <c r="H47" s="34"/>
-      <c r="I47" s="34"/>
-      <c r="J47" s="34"/>
-      <c r="K47" s="34"/>
-      <c r="L47" s="34"/>
-      <c r="M47" s="34"/>
-      <c r="N47" s="34"/>
-      <c r="O47" s="34"/>
-      <c r="P47" s="34"/>
+      <c r="A47" s="4"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="4"/>
+      <c r="H47" s="4"/>
+      <c r="I47" s="4"/>
+      <c r="J47" s="4"/>
+      <c r="K47" s="4"/>
+      <c r="L47" s="4"/>
+      <c r="M47" s="4"/>
+      <c r="N47" s="4"/>
+      <c r="O47" s="4"/>
+      <c r="P47" s="4"/>
     </row>
     <row r="48" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="34"/>
-      <c r="B48" s="34"/>
-      <c r="C48" s="34"/>
-      <c r="D48" s="34"/>
-      <c r="E48" s="34"/>
-      <c r="F48" s="34"/>
-      <c r="G48" s="34"/>
-      <c r="H48" s="34"/>
-      <c r="I48" s="34"/>
-      <c r="J48" s="34"/>
-      <c r="K48" s="34"/>
-      <c r="L48" s="34"/>
-      <c r="M48" s="34"/>
-      <c r="N48" s="34"/>
-      <c r="O48" s="34"/>
-      <c r="P48" s="34"/>
+      <c r="A48" s="4"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="4"/>
+      <c r="J48" s="4"/>
+      <c r="K48" s="4"/>
+      <c r="L48" s="4"/>
+      <c r="M48" s="4"/>
+      <c r="N48" s="4"/>
+      <c r="O48" s="4"/>
+      <c r="P48" s="4"/>
     </row>
     <row r="49" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="36"/>
-      <c r="B49" s="36"/>
-      <c r="C49" s="36"/>
-      <c r="D49" s="36"/>
-      <c r="E49" s="36"/>
-      <c r="F49" s="36"/>
-      <c r="G49" s="36"/>
-      <c r="H49" s="36"/>
-      <c r="I49" s="36"/>
-      <c r="J49" s="36"/>
-      <c r="K49" s="36"/>
-      <c r="L49" s="36"/>
-      <c r="M49" s="36"/>
-      <c r="N49" s="36"/>
-      <c r="O49" s="36"/>
-      <c r="P49" s="36"/>
+      <c r="A49" s="6"/>
+      <c r="B49" s="6"/>
+      <c r="C49" s="6"/>
+      <c r="D49" s="6"/>
+      <c r="E49" s="6"/>
+      <c r="F49" s="6"/>
+      <c r="G49" s="6"/>
+      <c r="H49" s="6"/>
+      <c r="I49" s="6"/>
+      <c r="J49" s="6"/>
+      <c r="K49" s="6"/>
+      <c r="L49" s="6"/>
+      <c r="M49" s="6"/>
+      <c r="N49" s="6"/>
+      <c r="O49" s="6"/>
+      <c r="P49" s="6"/>
     </row>
     <row r="50" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="36"/>
-      <c r="B50" s="36"/>
-      <c r="C50" s="36"/>
-      <c r="D50" s="36"/>
-      <c r="E50" s="36"/>
-      <c r="F50" s="36"/>
-      <c r="G50" s="36"/>
-      <c r="H50" s="36"/>
-      <c r="I50" s="36"/>
-      <c r="J50" s="36"/>
-      <c r="K50" s="36"/>
-      <c r="L50" s="36"/>
-      <c r="M50" s="36"/>
-      <c r="N50" s="36"/>
-      <c r="O50" s="36"/>
-      <c r="P50" s="36"/>
+      <c r="A50" s="6"/>
+      <c r="B50" s="6"/>
+      <c r="C50" s="6"/>
+      <c r="D50" s="6"/>
+      <c r="E50" s="6"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="6"/>
+      <c r="H50" s="6"/>
+      <c r="I50" s="6"/>
+      <c r="J50" s="6"/>
+      <c r="K50" s="6"/>
+      <c r="L50" s="6"/>
+      <c r="M50" s="6"/>
+      <c r="N50" s="6"/>
+      <c r="O50" s="6"/>
+      <c r="P50" s="6"/>
     </row>
     <row r="51" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="36"/>
-      <c r="B51" s="36"/>
-      <c r="C51" s="36"/>
-      <c r="D51" s="36"/>
-      <c r="E51" s="36"/>
-      <c r="F51" s="36"/>
-      <c r="G51" s="36"/>
-      <c r="H51" s="36"/>
-      <c r="I51" s="36"/>
-      <c r="J51" s="36"/>
-      <c r="K51" s="36"/>
-      <c r="L51" s="36"/>
-      <c r="M51" s="36"/>
-      <c r="N51" s="36"/>
-      <c r="O51" s="36"/>
-      <c r="P51" s="36"/>
+      <c r="A51" s="6"/>
+      <c r="B51" s="6"/>
+      <c r="C51" s="6"/>
+      <c r="D51" s="6"/>
+      <c r="E51" s="6"/>
+      <c r="F51" s="6"/>
+      <c r="G51" s="6"/>
+      <c r="H51" s="6"/>
+      <c r="I51" s="6"/>
+      <c r="J51" s="6"/>
+      <c r="K51" s="6"/>
+      <c r="L51" s="6"/>
+      <c r="M51" s="6"/>
+      <c r="N51" s="6"/>
+      <c r="O51" s="6"/>
+      <c r="P51" s="6"/>
     </row>
     <row r="52" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="36"/>
-      <c r="B52" s="36"/>
-      <c r="C52" s="36"/>
-      <c r="D52" s="36"/>
-      <c r="E52" s="36"/>
-      <c r="F52" s="36"/>
-      <c r="G52" s="36"/>
-      <c r="H52" s="36"/>
-      <c r="I52" s="36"/>
-      <c r="J52" s="36"/>
-      <c r="K52" s="36"/>
-      <c r="L52" s="36"/>
-      <c r="M52" s="36"/>
-      <c r="N52" s="36"/>
-      <c r="O52" s="36"/>
-      <c r="P52" s="36"/>
+      <c r="A52" s="6"/>
+      <c r="B52" s="6"/>
+      <c r="C52" s="6"/>
+      <c r="D52" s="6"/>
+      <c r="E52" s="6"/>
+      <c r="F52" s="6"/>
+      <c r="G52" s="6"/>
+      <c r="H52" s="6"/>
+      <c r="I52" s="6"/>
+      <c r="J52" s="6"/>
+      <c r="K52" s="6"/>
+      <c r="L52" s="6"/>
+      <c r="M52" s="6"/>
+      <c r="N52" s="6"/>
+      <c r="O52" s="6"/>
+      <c r="P52" s="6"/>
     </row>
     <row r="53" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="54" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>